<commit_message>
A written match report under the intro; Cavendish is not a keeper
- The landing page carries a three-paragraph report of the latest game, below
  the intro: the result and how it turned, who scored and how the shooting
  went, then the goalkeeping, defence and discipline. It is generated from the
  game's own numbers, so every game published gets one without anyone writing
  it, and every clause is guarded — a thin old workbook simply says less.
- Halftime now rides the season record so the report can use it.
- C3C Ian P. Cavendish is removed from the Denver game's Goalkeepers sheet at
  the owner's request. He faced one shot and saved it, so the keeper rows now
  account for 69 of the 70 shots Denver took; goals allowed are unchanged,
  because that shot was a save.

Probe 187 -> 189.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
+++ b/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
@@ -404,10 +404,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B17"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -552,26 +548,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R16"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="5.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-    <col min="5" max="5" width="9.83203125" customWidth="1"/>
-    <col min="6" max="6" width="9.83203125" customWidth="1"/>
-    <col min="7" max="7" width="9.83203125" customWidth="1"/>
-    <col min="8" max="8" width="9.83203125" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" customWidth="1"/>
-    <col min="10" max="10" width="9.83203125" customWidth="1"/>
-    <col min="11" max="11" width="9.83203125" customWidth="1"/>
-    <col min="12" max="12" width="9.83203125" customWidth="1"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1"/>
-    <col min="15" max="15" width="9.83203125" customWidth="1"/>
-    <col min="16" max="16" width="9.83203125" customWidth="1"/>
-    <col min="17" max="17" width="9.83203125" customWidth="1"/>
-    <col min="18" max="18" width="9.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1478,18 +1454,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1551,65 +1516,36 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B3" t="str">
-        <v>C3C Ian P. Cavendish</v>
+        <v>C1C Zachary D. Crane</v>
       </c>
       <c r="C3">
+        <v>41</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>26.7</v>
+      </c>
+      <c r="F3">
+        <v>22</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="str">
-        <v>C1C Zachary D. Crane</v>
-      </c>
-      <c r="C4">
-        <v>41</v>
-      </c>
-      <c r="D4">
-        <v>8</v>
-      </c>
-      <c r="E4">
-        <v>26.7</v>
-      </c>
-      <c r="F4">
-        <v>22</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1617,11 +1553,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1765,19 +1696,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K155"/>
-  <cols>
-    <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="5.83203125" customWidth="1"/>
-    <col min="3" max="3" width="7.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="4.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="7.83203125" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" customWidth="1"/>
-    <col min="11" max="11" width="8.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7214,19 +7132,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K64"/>
-  <cols>
-    <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="5.83203125" customWidth="1"/>
-    <col min="3" max="3" width="7.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="4.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="5.83203125" customWidth="1"/>
-    <col min="9" max="9" width="7.83203125" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" customWidth="1"/>
-    <col min="11" max="11" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9478,13 +9383,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="6.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>